<commit_message>
Milana AI trip search, regions improvements and discovery experience polish
Add compact /regions discovery page with mini trip previews, recommendations filtering and saved trips UX, plus region data and place photo updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/imports/places-filter.xlsx
+++ b/data/imports/places-filter.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15.88" customWidth="1" style="5" min="1" max="1"/>
@@ -4417,6 +4417,48 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>משק בגבעה גדרה</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>מרכז</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Offroad foundation, domain launch, media sync and platform improvements
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/imports/places-filter.xlsx
+++ b/data/imports/places-filter.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15.88" customWidth="1" style="5" min="1" max="1"/>
@@ -4418,44 +4418,128 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="0" t="inlineStr">
         <is>
           <t>משק בגבעה גדרה</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="0" t="inlineStr">
         <is>
           <t>מרכז</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>לא</t>
+      <c r="C96" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E96" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F96" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G96" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H96" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t>פארק אוטופיה</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t>השרון</t>
+        </is>
+      </c>
+      <c r="C97" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D97" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E97" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F97" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G97" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H97" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>בלאגן ביגור</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>צפון</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>כן</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add five North region stub trips from master sheet
Add coming-soon pages for עין איוב, עין מגדל, עין נון, תצפית הר הארי, and בית ג׳ן with synced filter tags and SEO-friendly slugs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/imports/places-filter.xlsx
+++ b/data/imports/places-filter.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15.88" customWidth="1" style="5" min="1" max="1"/>
@@ -4502,42 +4502,252 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="0" t="inlineStr">
         <is>
           <t>בלאגן ביגור</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="0" t="inlineStr">
         <is>
           <t>צפון</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
+      <c r="C98" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D98" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E98" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F98" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G98" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H98" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>עין איוב</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>צפון</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>עין מגדל</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>צפון</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>עין נון</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>צפון</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>תצפית הר הארי</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>צפון</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>בית ג׳ן</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>צפון</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
         <is>
           <t>כן</t>
         </is>

</xml_diff>

<commit_message>
Remove מצפה ארבל from project
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/imports/places-filter.xlsx
+++ b/data/imports/places-filter.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15.88" customWidth="1" style="5" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>מצפה ארבל</t>
+          <t>שמורת תל דן</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -482,12 +482,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -502,19 +502,19 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>שמורת תל דן</t>
+          <t>בריכת רם - מסעדה</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -544,19 +544,19 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>בריכת רם - מסעדה</t>
+          <t>חרמון</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -586,19 +586,19 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>חרמון</t>
+          <t>אגמון החולה</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>אגמון החולה</t>
+          <t>קיבוץ אפיקים</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -675,14 +675,14 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>קיבוץ אפיקים</t>
+          <t>נחל שופט</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -724,7 +724,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>נחל שופט</t>
+          <t>מעיין הסוסים</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>מעיין הסוסים</t>
+          <t>שמורת טבע בניאס</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -791,24 +791,24 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>שמורת טבע בניאס</t>
+          <t>מסעדת דג על הדן</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -850,7 +850,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>מסעדת דג על הדן</t>
+          <t>מפל תנור גבול לבנון</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -885,14 +885,14 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>מפל תנור גבול לבנון</t>
+          <t>פארק נחל קרת</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -934,7 +934,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>פארק נחל קרת</t>
+          <t>רוב רוי</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -976,7 +976,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>רוב רוי</t>
+          <t>נחל הקיבוצים</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1018,7 +1018,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>נחל הקיבוצים</t>
+          <t>נחל האסי</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1060,7 +1060,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>נחל האסי</t>
+          <t>חורשת גדעונה</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1102,17 +1102,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>חורשת גדעונה</t>
+          <t>רמת גן - ספארי</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1132,19 +1132,19 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>רמת גן - ספארי</t>
+          <t>פארק אריאל שרון</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1179,14 +1179,14 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>פארק אריאל שרון</t>
+          <t>פארק מים שפיים</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1196,12 +1196,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1221,14 +1221,14 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>פארק מים שפיים</t>
+          <t>פארק מים מודיעין</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1270,17 +1270,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>פארק מים מודיעין</t>
+          <t>פארק רעננה</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1305,14 +1305,14 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>פארק רעננה</t>
+          <t>נחל אלכסנדר</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1354,17 +1354,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>נחל אלכסנדר</t>
+          <t>לגעת בחיות</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1389,24 +1389,24 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>לגעת בחיות</t>
+          <t>חוף עתלית</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1426,19 +1426,19 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>חוף עתלית</t>
+          <t>חוף אולגה</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1480,7 +1480,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>חוף אולגה</t>
+          <t>מצפור ויקר</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1522,12 +1522,12 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>מצפור ויקר</t>
+          <t>שמורת טבע נחל שורק</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>שמורת טבע נחל שורק</t>
+          <t>הגבעות של נס ציונה</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -1606,17 +1606,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>הגבעות של נס ציונה</t>
+          <t>נחל תנינים</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1631,12 +1631,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1648,7 +1648,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>נחל תנינים</t>
+          <t>מעגן מיכאל פסל הלב</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -1690,12 +1690,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>מעגן מיכאל פסל הלב</t>
+          <t>שמורת פלמחים</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1705,12 +1705,12 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1732,7 +1732,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>שמורת פלמחים</t>
+          <t>תל אפק</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1762,34 +1762,34 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>תל אפק</t>
+          <t>גן החיות התנכי</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1816,7 +1816,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>גן החיות התנכי</t>
+          <t>אקווריום ישראל</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1858,12 +1858,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>אקווריום ישראל</t>
+          <t>פארק יטבתה</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1893,14 +1893,14 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>פארק יטבתה</t>
+          <t>ים המלח - חוף ביאניקני</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1935,14 +1935,14 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>ים המלח - חוף ביאניקני</t>
+          <t>מרינה אשקלון</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -1977,14 +1977,14 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>מרינה אשקלון</t>
+          <t>לונדע</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -2019,24 +2019,24 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>לונדע</t>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>בניאס</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>בניאס</t>
+          <t>שמורת טבע גמלא</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2078,12 +2078,12 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2110,7 +2110,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>שמורת טבע גמלא</t>
+          <t>יקב רמת הגולן</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2145,19 +2145,19 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>יקב רמת הגולן</t>
+          <t>מעיינות גיבתון</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2194,12 +2194,12 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>מעיינות גיבתון</t>
+          <t>יער צרעה</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2214,17 +2214,17 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2236,27 +2236,27 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>יער צרעה</t>
+          <t>חוף החשמל</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2278,7 +2278,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>חוף החשמל</t>
+          <t>תל גזר</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -2288,12 +2288,12 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -2303,12 +2303,12 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -2320,12 +2320,12 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>תל גזר</t>
+          <t>פארק קנדה</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2345,12 +2345,12 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -2362,22 +2362,22 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>פארק קנדה</t>
+          <t>עין פאשחה עיינות צוקים</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2397,14 +2397,14 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>עין פאשחה עיינות צוקים</t>
+          <t>אגם ניצנים</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2424,34 +2424,34 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>אגם ניצנים</t>
+          <t>עין לבן</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -2461,17 +2461,17 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2488,22 +2488,22 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>עין לבן</t>
+          <t>פארק אקולוגי הוד השרון</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -2530,17 +2530,17 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>פארק אקולוגי הוד השרון</t>
+          <t>המפל הנסתר פתח תקווה</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2555,12 +2555,12 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -2572,7 +2572,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>המפל הנסתר פתח תקווה</t>
+          <t>בית לאה</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2614,7 +2614,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>בית לאה</t>
+          <t>תחנת אבו רבאח</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -2656,12 +2656,12 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>תחנת אבו רבאח</t>
+          <t>פארק נחל לכיש</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -2681,12 +2681,12 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -2698,37 +2698,37 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>פארק נחל לכיש</t>
+          <t>יער המגינים</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -2740,22 +2740,22 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>יער המגינים</t>
+          <t>עין חרוד</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -2765,24 +2765,24 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>עין חרוד</t>
+          <t>עין מודע</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2817,14 +2817,14 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>עין מודע</t>
+          <t>נחל הקיבוצים</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>נחל הקיבוצים</t>
+          <t>כינרת</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -2891,12 +2891,12 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
@@ -2908,7 +2908,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>כינרת</t>
+          <t>גני חוגה</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -2943,14 +2943,14 @@
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>גני חוגה</t>
+          <t>סכר אלומות</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -2980,19 +2980,19 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>סכר אלומות</t>
+          <t>ראש הנקרה</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3002,12 +3002,12 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -3027,14 +3027,14 @@
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>ראש הנקרה</t>
+          <t>עין חרדלית</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
@@ -3059,24 +3059,24 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>עין חרדלית</t>
+          <t>החוף של מוש אכזיב</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -3091,22 +3091,22 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
@@ -3118,17 +3118,17 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>החוף של מוש אכזיב</t>
+          <t>קומראן</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -3153,14 +3153,14 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>קומראן</t>
+          <t>חאן עין גדי</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3202,7 +3202,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>חאן עין גדי</t>
+          <t>אמציה</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -3217,12 +3217,12 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -3237,14 +3237,14 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>אמציה</t>
+          <t>יער המלאכים</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -3259,22 +3259,22 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -3286,12 +3286,12 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>יער המלאכים</t>
+          <t>קלחים ומבוכים</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -3301,39 +3301,39 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>קלחים ומבוכים</t>
+          <t>גן לאומי מגדל צדק</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
@@ -3370,12 +3370,12 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>גן לאומי מגדל צדק</t>
+          <t>בת שלמה</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -3395,29 +3395,29 @@
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>בת שלמה</t>
+          <t>טל שחר</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3454,7 +3454,7 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>טל שחר</t>
+          <t>עיזה פזיזה</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -3496,7 +3496,7 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>עיזה פזיזה</t>
+          <t>משמר דוד</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
@@ -3521,12 +3521,12 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
@@ -3538,12 +3538,12 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>משמר דוד</t>
+          <t>בית גוברין</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -3573,14 +3573,14 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>בית גוברין</t>
+          <t>נחל דוד</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
@@ -3605,12 +3605,12 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -3622,17 +3622,17 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>נחל דוד</t>
+          <t>מוזיאון הילדים חולון</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -3664,17 +3664,17 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>מוזיאון הילדים חולון</t>
+          <t>עין חמד</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -3706,22 +3706,22 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>עין חמד</t>
+          <t>נוף איילון</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -3736,19 +3736,19 @@
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>נוף איילון</t>
+          <t>פארק בריטניה</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -3768,12 +3768,12 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -3790,12 +3790,12 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>פארק בריטניה</t>
+          <t>בתרונות רוחמה</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -3832,22 +3832,22 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>בתרונות רוחמה</t>
+          <t>ברבטבע</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -3857,12 +3857,12 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
@@ -3874,7 +3874,7 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>ברבטבע</t>
+          <t>רבדים</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
@@ -3916,7 +3916,7 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>רבדים</t>
+          <t>גבעת הרקפות</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -3926,12 +3926,12 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -3958,22 +3958,22 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>גבעת הרקפות</t>
+          <t>עין בוקק</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
@@ -4000,22 +4000,22 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>עין בוקק</t>
+          <t>עמק האלה</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
@@ -4042,17 +4042,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>עמק האלה</t>
+          <t>מאגר בית זית</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -4084,7 +4084,7 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>מאגר בית זית</t>
+          <t>הסטף</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
@@ -4126,12 +4126,12 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>הסטף</t>
+          <t>תל חדיד</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
@@ -4168,7 +4168,7 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>תל חדיד</t>
+          <t>מצפה אלון</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -4193,12 +4193,12 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -4210,12 +4210,12 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>מצפה אלון</t>
+          <t>מדבריום</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -4245,24 +4245,24 @@
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>מדבריום</t>
+          <t>עין ורדא</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -4277,24 +4277,24 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>עין ורדא</t>
+          <t>יער בן שמן</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -4304,17 +4304,17 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
@@ -4334,42 +4334,42 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>יער בן שמן</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>מרכז</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="E94" s="4" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="F94" s="4" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="G94" s="4" t="inlineStr">
-        <is>
-          <t>חלקי</t>
-        </is>
-      </c>
-      <c r="H94" s="4" t="inlineStr">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t>חוף מעגן מיכאל</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
+          <t>השרון</t>
+        </is>
+      </c>
+      <c r="C94" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D94" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="E94" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F94" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G94" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H94" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
@@ -4378,22 +4378,22 @@
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t>חוף מעגן מיכאל</t>
+          <t>משק בגבעה גדרה</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D95" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E95" s="0" t="inlineStr">
@@ -4413,19 +4413,19 @@
       </c>
       <c r="H95" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="0" t="inlineStr">
         <is>
-          <t>משק בגבעה גדרה</t>
+          <t>פארק אוטופיה</t>
         </is>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
@@ -4462,17 +4462,17 @@
     <row r="97">
       <c r="A97" s="0" t="inlineStr">
         <is>
-          <t>פארק אוטופיה</t>
+          <t>בלאגן ביגור</t>
         </is>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D97" s="0" t="inlineStr">
@@ -4497,14 +4497,14 @@
       </c>
       <c r="H97" s="0" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t>בלאגן ביגור</t>
+          <t>עין איוב</t>
         </is>
       </c>
       <c r="B98" s="0" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H98" s="0" t="inlineStr">
@@ -4544,210 +4544,168 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>עין איוב</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t>עין מגדל</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
         <is>
           <t>צפון</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
+      <c r="C99" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D99" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E99" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F99" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G99" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H99" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>עין מגדל</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
+      <c r="A100" s="0" t="inlineStr">
+        <is>
+          <t>עין נון</t>
+        </is>
+      </c>
+      <c r="B100" s="0" t="inlineStr">
         <is>
           <t>צפון</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
+      <c r="C100" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D100" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="E100" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F100" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G100" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H100" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>עין נון</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t>תצפית הר הארי</t>
+        </is>
+      </c>
+      <c r="B101" s="0" t="inlineStr">
         <is>
           <t>צפון</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
+      <c r="C101" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D101" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="E101" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F101" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G101" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H101" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>תצפית הר הארי</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
+      <c r="A102" s="0" t="inlineStr">
+        <is>
+          <t>בית ג׳ן</t>
+        </is>
+      </c>
+      <c r="B102" s="0" t="inlineStr">
         <is>
           <t>צפון</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>בית ג׳ן</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
+      <c r="C102" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="D102" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="E102" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F102" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G102" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H102" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>

</xml_diff>

<commit_message>
Publish approved north trip content and data cleanup.
Integrate full pages for Banias, Agmon HaHula, Maayan HaSusim, Tel Dan waterfall, Nahal Nekarot, Rob Roy, Nahal HaKibbutzim, Nahal HaAsi, Gdona grove, Gamla, and Ein Harod; remove duplicate Banias stub, sync filter tags and photos, and fix duplicate React keys in trip experience paragraphs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/imports/places-filter.xlsx
+++ b/data/imports/places-filter.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15.88" customWidth="1" style="5" min="1" max="1"/>
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>שמורת טבע בניאס</t>
+          <t>שמורת הטבע בניאס</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>בניאס</t>
+          <t>שמורת טבע גמלא</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2036,12 +2036,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>שמורת טבע גמלא</t>
+          <t>יקב רמת הגולן</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2103,19 +2103,19 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>יקב רמת הגולן</t>
+          <t>מעיינות גיבתון</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2152,12 +2152,12 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>מעיינות גיבתון</t>
+          <t>יער צרעה</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2172,17 +2172,17 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2194,27 +2194,27 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>יער צרעה</t>
+          <t>חוף החשמל</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2236,7 +2236,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>חוף החשמל</t>
+          <t>תל גזר</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2246,12 +2246,12 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2278,12 +2278,12 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>תל גזר</t>
+          <t>פארק קנדה</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -2303,12 +2303,12 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -2320,22 +2320,22 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>פארק קנדה</t>
+          <t>עין פאשחה עיינות צוקים</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2355,14 +2355,14 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>עין פאשחה עיינות צוקים</t>
+          <t>אגם ניצנים</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -2382,34 +2382,34 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>אגם ניצנים</t>
+          <t>עין לבן</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -2419,17 +2419,17 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2446,22 +2446,22 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>עין לבן</t>
+          <t>פארק אקולוגי הוד השרון</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -2488,17 +2488,17 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>פארק אקולוגי הוד השרון</t>
+          <t>המפל הנסתר פתח תקווה</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -2513,12 +2513,12 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -2530,7 +2530,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>המפל הנסתר פתח תקווה</t>
+          <t>בית לאה</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -2572,7 +2572,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>בית לאה</t>
+          <t>תחנת אבו רבאח</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2614,12 +2614,12 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>תחנת אבו רבאח</t>
+          <t>פארק נחל לכיש</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -2639,12 +2639,12 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -2656,37 +2656,37 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>פארק נחל לכיש</t>
+          <t>יער המגינים</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -2698,17 +2698,17 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>יער המגינים</t>
+          <t>עין חרוד</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2723,24 +2723,24 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>עין חרוד</t>
+          <t>עין מודע</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -2775,14 +2775,14 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>עין מודע</t>
+          <t>נחל הקיבוצים</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -2824,7 +2824,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>נחל הקיבוצים</t>
+          <t>כינרת</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -2849,12 +2849,12 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>כינרת</t>
+          <t>גני חוגה</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -2901,14 +2901,14 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>גני חוגה</t>
+          <t>סכר אלומות</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -2938,19 +2938,19 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>סכר אלומות</t>
+          <t>ראש הנקרה</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -2960,12 +2960,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -2985,14 +2985,14 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>ראש הנקרה</t>
+          <t>עין חרדלית</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3002,12 +3002,12 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -3017,24 +3017,24 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>עין חרדלית</t>
+          <t>החוף של מוש אכזיב</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -3049,22 +3049,22 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -3076,17 +3076,17 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>החוף של מוש אכזיב</t>
+          <t>קומראן</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -3111,14 +3111,14 @@
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>קומראן</t>
+          <t>חאן עין גדי</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -3160,7 +3160,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>חאן עין גדי</t>
+          <t>אמציה</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3175,12 +3175,12 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3195,14 +3195,14 @@
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>אמציה</t>
+          <t>יער המלאכים</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -3217,22 +3217,22 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
@@ -3244,12 +3244,12 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>יער המלאכים</t>
+          <t>קלחים ומבוכים</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -3259,39 +3259,39 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>קלחים ומבוכים</t>
+          <t>גן לאומי מגדל צדק</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
@@ -3328,12 +3328,12 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>גן לאומי מגדל צדק</t>
+          <t>בת שלמה</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -3353,29 +3353,29 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>בת שלמה</t>
+          <t>טל שחר</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>צפון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -3412,7 +3412,7 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>טל שחר</t>
+          <t>עיזה פזיזה</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -3454,7 +3454,7 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>עיזה פזיזה</t>
+          <t>משמר דוד</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -3479,12 +3479,12 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
@@ -3496,12 +3496,12 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>משמר דוד</t>
+          <t>בית גוברין</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -3531,14 +3531,14 @@
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>בית גוברין</t>
+          <t>נחל דוד</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -3548,12 +3548,12 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -3563,12 +3563,12 @@
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -3580,17 +3580,17 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>נחל דוד</t>
+          <t>מוזיאון הילדים חולון</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -3622,17 +3622,17 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>מוזיאון הילדים חולון</t>
+          <t>עין חמד</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -3664,22 +3664,22 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>עין חמד</t>
+          <t>נוף איילון</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -3694,19 +3694,19 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>נוף איילון</t>
+          <t>פארק בריטניה</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -3726,12 +3726,12 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
@@ -3748,12 +3748,12 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>פארק בריטניה</t>
+          <t>בתרונות רוחמה</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
@@ -3790,22 +3790,22 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>בתרונות רוחמה</t>
+          <t>ברבטבע</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -3815,12 +3815,12 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -3832,7 +3832,7 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>ברבטבע</t>
+          <t>רבדים</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -3857,12 +3857,12 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
@@ -3874,7 +3874,7 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>רבדים</t>
+          <t>גבעת הרקפות</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -3884,12 +3884,12 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -3916,22 +3916,22 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>גבעת הרקפות</t>
+          <t>עין בוקק</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
@@ -3958,22 +3958,22 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>עין בוקק</t>
+          <t>עמק האלה</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
@@ -4000,17 +4000,17 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>עמק האלה</t>
+          <t>מאגר בית זית</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
@@ -4042,7 +4042,7 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>מאגר בית זית</t>
+          <t>הסטף</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>חלקי</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -4084,12 +4084,12 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>הסטף</t>
+          <t>תל חדיד</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
@@ -4126,7 +4126,7 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>תל חדיד</t>
+          <t>מצפה אלון</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -4151,12 +4151,12 @@
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
@@ -4168,12 +4168,12 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>מצפה אלון</t>
+          <t>מדבריום</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -4203,24 +4203,24 @@
       </c>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>מדבריום</t>
+          <t>עין ורדא</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -4235,24 +4235,24 @@
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>עין ורדא</t>
+          <t>יער בן שמן</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -4262,17 +4262,17 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
@@ -4292,42 +4292,42 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>יער בן שמן</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>מרכז</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="F93" s="4" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="G93" s="4" t="inlineStr">
-        <is>
-          <t>חלקי</t>
-        </is>
-      </c>
-      <c r="H93" s="4" t="inlineStr">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t>חוף מעגן מיכאל</t>
+        </is>
+      </c>
+      <c r="B93" s="0" t="inlineStr">
+        <is>
+          <t>השרון</t>
+        </is>
+      </c>
+      <c r="C93" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D93" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="E93" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="F93" s="0" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="G93" s="0" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="H93" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
@@ -4336,22 +4336,22 @@
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t>חוף מעגן מיכאל</t>
+          <t>משק בגבעה גדרה</t>
         </is>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="E94" s="0" t="inlineStr">
@@ -4371,19 +4371,19 @@
       </c>
       <c r="H94" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t>משק בגבעה גדרה</t>
+          <t>פארק אוטופיה</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>השרון</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
@@ -4420,17 +4420,17 @@
     <row r="96">
       <c r="A96" s="0" t="inlineStr">
         <is>
-          <t>פארק אוטופיה</t>
+          <t>בלאגן ביגור</t>
         </is>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>השרון</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="D96" s="0" t="inlineStr">
@@ -4455,14 +4455,14 @@
       </c>
       <c r="H96" s="0" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="0" t="inlineStr">
         <is>
-          <t>בלאגן ביגור</t>
+          <t>עין איוב</t>
         </is>
       </c>
       <c r="B97" s="0" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -4504,7 +4504,7 @@
     <row r="98">
       <c r="A98" s="0" t="inlineStr">
         <is>
-          <t>עין איוב</t>
+          <t>עין מגדל</t>
         </is>
       </c>
       <c r="B98" s="0" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="H98" s="0" t="inlineStr">
@@ -4546,7 +4546,7 @@
     <row r="99">
       <c r="A99" s="0" t="inlineStr">
         <is>
-          <t>עין מגדל</t>
+          <t>עין נון</t>
         </is>
       </c>
       <c r="B99" s="0" t="inlineStr">
@@ -4588,7 +4588,7 @@
     <row r="100">
       <c r="A100" s="0" t="inlineStr">
         <is>
-          <t>עין נון</t>
+          <t>תצפית הר הארי</t>
         </is>
       </c>
       <c r="B100" s="0" t="inlineStr">
@@ -4598,12 +4598,12 @@
       </c>
       <c r="C100" s="0" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="D100" s="0" t="inlineStr">
         <is>
-          <t>לא</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="E100" s="0" t="inlineStr">
@@ -4630,7 +4630,7 @@
     <row r="101">
       <c r="A101" s="0" t="inlineStr">
         <is>
-          <t>תצפית הר הארי</t>
+          <t>בית ג׳ן</t>
         </is>
       </c>
       <c r="B101" s="0" t="inlineStr">
@@ -4664,48 +4664,6 @@
         </is>
       </c>
       <c r="H101" s="0" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="0" t="inlineStr">
-        <is>
-          <t>בית ג׳ן</t>
-        </is>
-      </c>
-      <c r="B102" s="0" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="C102" s="0" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="D102" s="0" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="E102" s="0" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="F102" s="0" t="inlineStr">
-        <is>
-          <t>לא</t>
-        </is>
-      </c>
-      <c r="G102" s="0" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="H102" s="0" t="inlineStr">
         <is>
           <t>כן</t>
         </is>

</xml_diff>

<commit_message>
Add approved North trip content batch (Head of Hanikra, Ein Hardalit, Mosh Beach Achziv, Bat Shlomo and related updates).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/imports/places-filter.xlsx
+++ b/data/imports/places-filter.xlsx
@@ -3017,7 +3017,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לא</t>
         </is>
       </c>
     </row>

</xml_diff>